<commit_message>
Improve workbook labeling and language detection
</commit_message>
<xml_diff>
--- a/excel/fmcg-inventory-control-tower.xlsx
+++ b/excel/fmcg-inventory-control-tower.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Tower" sheetId="1" r:id="Re88f06362c3a430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Policy" sheetId="2" r:id="Rac008d9b30a34d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABC-XYZ Matrix" sheetId="3" r:id="R4a1af6dac45e44cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand History" sheetId="4" r:id="R948d67c91b1e4a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="5" r:id="R617ff3746f2f4dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Notes" sheetId="6" r:id="R6304ba18525642ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Tower" sheetId="1" r:id="Re794e3c54d794d71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Policy" sheetId="2" r:id="Rdc02cddc66be4d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABC-XYZ Matrix" sheetId="3" r:id="Rb1cb55d2f29c4f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand History" sheetId="4" r:id="R91c2409703b64389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="5" r:id="Ree460aff80c14e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Notes" sheetId="6" r:id="Ra549a765928d4582"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1101,7 +1101,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf7c4606c9ce94d17"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R97598fc5946e4b8c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1131,7 +1131,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rae5051122ca042b2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0c75291470e432e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1449,7 +1449,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="71" t="str">
-        <x:v>Synthetic 36-SKU portfolio | Formula-driven Excel model | Python and SQL reconciliation</x:v>
+        <x:v>Synthetic 36-SKU model | Formula-driven Excel analysis | Python and SQL reconciliation</x:v>
       </x:c>
       <x:c r="B3" s="71"/>
       <x:c r="C3" s="71"/>
@@ -1791,7 +1791,7 @@
     <x:mergeCell ref="A31:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56dcd52e6a844ecc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94323122bcc84b04"/>
 </x:worksheet>
 </file>
 
@@ -5654,7 +5654,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82fc6c61d5844a18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3c1ef6bbe342d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8861,7 +8861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad7c2f9e9ea1437e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cde6d3a9586475f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Tighten project copy and artifact labels
</commit_message>
<xml_diff>
--- a/excel/fmcg-inventory-control-tower.xlsx
+++ b/excel/fmcg-inventory-control-tower.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Tower" sheetId="1" r:id="Re794e3c54d794d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Policy" sheetId="2" r:id="Rdc02cddc66be4d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABC-XYZ Matrix" sheetId="3" r:id="Rb1cb55d2f29c4f48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand History" sheetId="4" r:id="R91c2409703b64389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="5" r:id="Ree460aff80c14e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Notes" sheetId="6" r:id="Ra549a765928d4582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Tower" sheetId="1" r:id="R69918325393e4de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU Policy" sheetId="2" r:id="Rc9de3d51838a4b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ABC-XYZ Matrix" sheetId="3" r:id="R835a7f1447314974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand History" sheetId="4" r:id="R562f99d613864257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="5" r:id="Rb36a332bffb348fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Notes" sheetId="6" r:id="R3eb5e9e94dca402c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1101,7 +1101,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R97598fc5946e4b8c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0f0405c8a314e64"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1131,7 +1131,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0c75291470e432e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra95105cad6b04380"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1449,7 +1449,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="71" t="str">
-        <x:v>Synthetic 36-SKU model | Formula-driven Excel analysis | Python and SQL reconciliation</x:v>
+        <x:v>36 SKUs | 24 months | Excel model with Python and SQL checks</x:v>
       </x:c>
       <x:c r="B3" s="71"/>
       <x:c r="C3" s="71"/>
@@ -1609,45 +1609,45 @@
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="B9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="C9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="D9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="E9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="F9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="H9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="I9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="J9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="K9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
       <x:c r="L9" s="39" t="str">
-        <x:v>Operating call</x:v>
+        <x:v>Today's queue</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="143" t="str">
-        <x:v>Protect service first: 6 SKUs sit below expected lead-time demand in the fixed dataset.</x:v>
+        <x:v>Check service first: 6 SKUs sit below expected lead-time demand.</x:v>
       </x:c>
       <x:c r="B10" s="144"/>
       <x:c r="C10" s="144"/>
@@ -1726,7 +1726,7 @@
     <x:row r="30" ht="23" customHeight="1"/>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="169" t="str">
-        <x:v>Decision note: potential release is a review queue, not an automatic disposal instruction. Filter SKU Policy by Risk Status, Recommended Order or Potential Release to work the exceptions.</x:v>
+        <x:v>Potential release is a planner review queue. Filter SKU Policy by Risk Status, Recommended Order or Potential Release to work the exceptions.</x:v>
       </x:c>
       <x:c r="B31" s="170"/>
       <x:c r="C31" s="170"/>
@@ -1791,7 +1791,7 @@
     <x:mergeCell ref="A31:L33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94323122bcc84b04"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R468e60e8654c42cc"/>
 </x:worksheet>
 </file>
 
@@ -5654,7 +5654,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3c1ef6bbe342d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re76f3bb579434e9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5952,7 +5952,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Monthly demand history | 24 months | synthetic units</x:v>
+        <x:v>Monthly demand history | 24 months</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -8861,7 +8861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cde6d3a9586475f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55aa4a5b755c48e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9031,7 +9031,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Data notes and audit trail</x:v>
+        <x:v>Data notes and model logic</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -9060,7 +9060,7 @@
         <x:v>Data status</x:v>
       </x:c>
       <x:c r="B5" s="54" t="str">
-        <x:v>Synthetic. No employer, client, retailer or supplier records are used.</x:v>
+        <x:v>Generated practice data; assumptions are visible in this workbook and the Python script.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">

</xml_diff>